<commit_message>
Updates for initial release
</commit_message>
<xml_diff>
--- a/pcb/touched_out_synth_bom.xlsx
+++ b/pcb/touched_out_synth_bom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bloemerk\Desktop\synth\synth\TouchedOutSynth\pcb\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rache\Desktop\Future Pedals\TouchedOutSynth\pcb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B288D8A-1D4A-4268-B59A-E52A6A3B3435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D824CF56-58DB-4BDE-804C-254E3F4D90B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12210" yWindow="4275" windowWidth="15150" windowHeight="11220" xr2:uid="{1662CF9F-7921-4EE8-BA4B-5A0F10701ADA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1662CF9F-7921-4EE8-BA4B-5A0F10701ADA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Part</t>
   </si>
@@ -74,9 +74,6 @@
     <t>LED</t>
   </si>
   <si>
-    <t>Resistor</t>
-  </si>
-  <si>
     <t>1/8" Jack</t>
   </si>
   <si>
@@ -108,13 +105,22 @@
   </si>
   <si>
     <t>https://lovemyswitches.com/taiway-sub-mini-spdt-on-on-switch-solder-lug-short-shaft/</t>
+  </si>
+  <si>
+    <t>https://www.taydaelectronics.com/pj-320a-3-5-mm-audio-socket-through-hole-pcb-silver-plated.html</t>
+  </si>
+  <si>
+    <t>10 ohm Resistor</t>
+  </si>
+  <si>
+    <t>33 ohm Resistor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -489,15 +495,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AE929D5-FB56-4C4B-982F-949FBB44FC2F}">
   <dimension ref="A2:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" customWidth="1"/>
+    <col min="1" max="1" width="29.375" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" customWidth="1"/>
-    <col min="4" max="4" width="72.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.875" customWidth="1"/>
+    <col min="4" max="4" width="72.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="15">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -511,7 +517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -519,10 +525,10 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -530,10 +536,10 @@
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -541,10 +547,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -552,13 +558,13 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -566,10 +572,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -577,29 +583,32 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9">
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -607,7 +616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -615,25 +624,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>1</v>

</xml_diff>